<commit_message>
#5 Fresh Deliverables after modifications in Routing: Peripherals needs to be entered in BOM.
</commit_message>
<xml_diff>
--- a/Design_Files/BOM/Client_BOM.xlsx
+++ b/Design_Files/BOM/Client_BOM.xlsx
@@ -1,20 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LiberDB\Documents\GitHub\michaelquartey-sonographydevice-hw\Design_Files\BOM\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="19635" windowHeight="7650"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19635" windowHeight="7650"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="144525"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="318">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="319">
   <si>
     <t>#</t>
   </si>
@@ -964,23 +969,20 @@
     <t>Transducer(TX/RX)socket</t>
   </si>
   <si>
-    <t>Battery</t>
-  </si>
-  <si>
-    <t>ultrasound-gel for sonography</t>
+    <t>9V Battery</t>
+  </si>
+  <si>
+    <t>Gel for sonography/ultrasound</t>
+  </si>
+  <si>
+    <t>Gel to apply on human body before sonology procedure.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9">
-  <numFmts count="4">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="30">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1065,147 +1067,16 @@
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1230,194 +1101,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="22">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -1570,253 +1255,14 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="14" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="8" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1861,19 +1307,16 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1917,68 +1360,31 @@
       <alignment horizontal="left" vertical="top"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="49">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
-    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
-    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
-    <cellStyle name="Note" xfId="8" builtinId="10"/>
-    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
-    <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Input" xfId="16" builtinId="20"/>
-    <cellStyle name="Output" xfId="17" builtinId="21"/>
-    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
-    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
-    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
-    <cellStyle name="Total" xfId="21" builtinId="25"/>
-    <cellStyle name="Good" xfId="22" builtinId="26"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
-    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
-      <color rgb="0003A4CB"/>
-      <color rgb="002CD0B2"/>
+      <color rgb="FF03A4CB"/>
+      <color rgb="FF2CD0B2"/>
     </mruColors>
   </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -2236,25 +1642,26 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:M69"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="3.14285714285714" style="2" customWidth="1"/>
-    <col min="3" max="3" width="18.7142857142857" style="2" customWidth="1"/>
+    <col min="2" max="2" width="3.140625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" style="2" customWidth="1"/>
     <col min="4" max="4" width="36" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="26.5714285714286" customWidth="1"/>
-    <col min="7" max="7" width="33.4285714285714" customWidth="1"/>
-    <col min="8" max="8" width="21.4285714285714" customWidth="1"/>
-    <col min="9" max="9" width="17.8571428571429" customWidth="1"/>
-    <col min="10" max="10" width="16.7142857142857" customWidth="1"/>
-    <col min="11" max="12" width="29.4285714285714" customWidth="1"/>
+    <col min="6" max="6" width="26.5703125" customWidth="1"/>
+    <col min="7" max="7" width="33.42578125" customWidth="1"/>
+    <col min="8" max="8" width="21.42578125" customWidth="1"/>
+    <col min="9" max="9" width="17.85546875" customWidth="1"/>
+    <col min="10" max="10" width="16.7109375" customWidth="1"/>
+    <col min="11" max="12" width="29.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -2266,12 +1673,12 @@
       <c r="F1" s="5"/>
       <c r="G1" s="5"/>
       <c r="H1" s="5"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-    </row>
-    <row r="2" ht="15.75" spans="1:12">
+      <c r="I1" s="34"/>
+      <c r="J1" s="34"/>
+      <c r="K1" s="34"/>
+      <c r="L1" s="34"/>
+    </row>
+    <row r="2" spans="1:12">
       <c r="A2" s="3"/>
       <c r="B2" s="6" t="s">
         <v>0</v>
@@ -2310,7 +1717,7 @@
     <row r="3" spans="1:12">
       <c r="A3" s="3"/>
       <c r="B3" s="8">
-        <f>ROW(B3)-ROW($B$2)</f>
+        <f t="shared" ref="B3:B34" si="0">ROW(B3)-ROW($B$2)</f>
         <v>1</v>
       </c>
       <c r="C3" s="9" t="s">
@@ -2340,10 +1747,10 @@
       <c r="K3" s="10"/>
       <c r="L3" s="10"/>
     </row>
-    <row r="4" ht="24.75" spans="1:12">
+    <row r="4" spans="1:12" ht="24">
       <c r="A4" s="3"/>
       <c r="B4" s="8">
-        <f>ROW(B4)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="C4" s="12" t="s">
@@ -2376,7 +1783,7 @@
     <row r="5" spans="1:12">
       <c r="A5" s="3"/>
       <c r="B5" s="8">
-        <f>ROW(B5)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="C5" s="9" t="s">
@@ -2406,10 +1813,10 @@
       <c r="K5" s="10"/>
       <c r="L5" s="10"/>
     </row>
-    <row r="6" ht="24.75" spans="1:12">
+    <row r="6" spans="1:12" ht="24">
       <c r="A6" s="3"/>
       <c r="B6" s="8">
-        <f>ROW(B6)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="C6" s="12" t="s">
@@ -2439,10 +1846,10 @@
       <c r="K6" s="13"/>
       <c r="L6" s="13"/>
     </row>
-    <row r="7" ht="36.75" spans="1:12">
+    <row r="7" spans="1:12" ht="36">
       <c r="A7" s="3"/>
       <c r="B7" s="8">
-        <f>ROW(B7)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="C7" s="9" t="s">
@@ -2475,7 +1882,7 @@
     <row r="8" spans="1:12">
       <c r="A8" s="3"/>
       <c r="B8" s="8">
-        <f>ROW(B8)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="C8" s="12" t="s">
@@ -2508,7 +1915,7 @@
     <row r="9" spans="1:12">
       <c r="A9" s="3"/>
       <c r="B9" s="8">
-        <f>ROW(B9)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="C9" s="9" t="s">
@@ -2541,7 +1948,7 @@
     <row r="10" spans="1:12">
       <c r="A10" s="3"/>
       <c r="B10" s="8">
-        <f>ROW(B10)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="C10" s="12" t="s">
@@ -2571,10 +1978,10 @@
       <c r="K10" s="13"/>
       <c r="L10" s="13"/>
     </row>
-    <row r="11" ht="36.75" spans="1:12">
+    <row r="11" spans="1:12" ht="36">
       <c r="A11" s="3"/>
       <c r="B11" s="8">
-        <f>ROW(B11)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="C11" s="9" t="s">
@@ -2604,10 +2011,10 @@
       <c r="K11" s="10"/>
       <c r="L11" s="10"/>
     </row>
-    <row r="12" ht="36.75" spans="1:12">
+    <row r="12" spans="1:12" ht="36">
       <c r="A12" s="3"/>
       <c r="B12" s="8">
-        <f>ROW(B12)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="C12" s="12" t="s">
@@ -2637,10 +2044,10 @@
       <c r="K12" s="13"/>
       <c r="L12" s="13"/>
     </row>
-    <row r="13" ht="24.75" spans="1:12">
+    <row r="13" spans="1:12" ht="24">
       <c r="A13" s="3"/>
       <c r="B13" s="8">
-        <f>ROW(B13)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="C13" s="9" t="s">
@@ -2670,10 +2077,10 @@
       <c r="K13" s="10"/>
       <c r="L13" s="10"/>
     </row>
-    <row r="14" ht="36.75" spans="1:12">
+    <row r="14" spans="1:12" ht="36">
       <c r="A14" s="3"/>
       <c r="B14" s="8">
-        <f>ROW(B14)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="C14" s="12" t="s">
@@ -2703,10 +2110,10 @@
       <c r="K14" s="13"/>
       <c r="L14" s="13"/>
     </row>
-    <row r="15" ht="36.75" spans="1:12">
+    <row r="15" spans="1:12" ht="36">
       <c r="A15" s="3"/>
       <c r="B15" s="8">
-        <f>ROW(B15)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="C15" s="9" t="s">
@@ -2736,10 +2143,10 @@
       <c r="K15" s="10"/>
       <c r="L15" s="10"/>
     </row>
-    <row r="16" ht="24.75" spans="1:12">
+    <row r="16" spans="1:12" ht="24">
       <c r="A16" s="3"/>
       <c r="B16" s="8">
-        <f>ROW(B16)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="C16" s="12" t="s">
@@ -2769,10 +2176,10 @@
       <c r="K16" s="13"/>
       <c r="L16" s="13"/>
     </row>
-    <row r="17" ht="26.25" spans="1:12">
+    <row r="17" spans="1:12" ht="25.5">
       <c r="A17" s="3"/>
       <c r="B17" s="8">
-        <f>ROW(B17)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="C17" s="9" t="s">
@@ -2802,10 +2209,10 @@
       <c r="K17" s="10"/>
       <c r="L17" s="10"/>
     </row>
-    <row r="18" ht="24.75" spans="1:12">
+    <row r="18" spans="1:12" ht="36">
       <c r="A18" s="3"/>
       <c r="B18" s="8">
-        <f>ROW(B18)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="C18" s="12" t="s">
@@ -2835,10 +2242,10 @@
       <c r="K18" s="13"/>
       <c r="L18" s="13"/>
     </row>
-    <row r="19" ht="24.75" spans="1:12">
+    <row r="19" spans="1:12" ht="24">
       <c r="A19" s="3"/>
       <c r="B19" s="8">
-        <f>ROW(B19)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="C19" s="9" t="s">
@@ -2868,10 +2275,10 @@
       <c r="K19" s="10"/>
       <c r="L19" s="10"/>
     </row>
-    <row r="20" ht="36.75" spans="1:12">
+    <row r="20" spans="1:12" ht="36">
       <c r="A20" s="3"/>
       <c r="B20" s="8">
-        <f>ROW(B20)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="C20" s="12" t="s">
@@ -2901,10 +2308,10 @@
       <c r="K20" s="13"/>
       <c r="L20" s="13"/>
     </row>
-    <row r="21" ht="24.75" spans="1:12">
+    <row r="21" spans="1:12" ht="24">
       <c r="A21" s="3"/>
       <c r="B21" s="8">
-        <f>ROW(B21)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>19</v>
       </c>
       <c r="C21" s="9" t="s">
@@ -2934,10 +2341,10 @@
       <c r="K21" s="10"/>
       <c r="L21" s="10"/>
     </row>
-    <row r="22" ht="48.75" spans="1:12">
+    <row r="22" spans="1:12" ht="60">
       <c r="A22" s="3"/>
       <c r="B22" s="8">
-        <f>ROW(B22)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="C22" s="12" t="s">
@@ -2964,15 +2371,15 @@
       <c r="J22" s="15">
         <v>1</v>
       </c>
-      <c r="K22" s="19"/>
-      <c r="L22" s="20" t="s">
+      <c r="K22" s="18"/>
+      <c r="L22" s="19" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="23" ht="15.75" spans="1:12">
+    <row r="23" spans="1:12">
       <c r="A23" s="3"/>
       <c r="B23" s="8">
-        <f>ROW(B23)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
       <c r="C23" s="9" t="s">
@@ -3002,10 +2409,10 @@
       <c r="K23" s="10"/>
       <c r="L23" s="10"/>
     </row>
-    <row r="24" ht="24.75" spans="1:12">
+    <row r="24" spans="1:12" ht="36">
       <c r="A24" s="3"/>
       <c r="B24" s="8">
-        <f>ROW(B24)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>22</v>
       </c>
       <c r="C24" s="12" t="s">
@@ -3038,7 +2445,7 @@
     <row r="25" spans="1:12">
       <c r="A25" s="3"/>
       <c r="B25" s="8">
-        <f>ROW(B25)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
       <c r="C25" s="9" t="s">
@@ -3068,10 +2475,10 @@
       <c r="K25" s="10"/>
       <c r="L25" s="10"/>
     </row>
-    <row r="26" ht="15.75" spans="1:12">
+    <row r="26" spans="1:12">
       <c r="A26" s="3"/>
       <c r="B26" s="8">
-        <f>ROW(B26)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="C26" s="12" t="s">
@@ -3101,10 +2508,10 @@
       <c r="K26" s="13"/>
       <c r="L26" s="13"/>
     </row>
-    <row r="27" ht="24.75" spans="1:12">
+    <row r="27" spans="1:12" ht="24">
       <c r="A27" s="3"/>
       <c r="B27" s="8">
-        <f>ROW(B27)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>25</v>
       </c>
       <c r="C27" s="12" t="s">
@@ -3134,10 +2541,10 @@
       <c r="K27" s="10"/>
       <c r="L27" s="10"/>
     </row>
-    <row r="28" ht="36.75" spans="1:12">
+    <row r="28" spans="1:12" ht="36">
       <c r="A28" s="3"/>
       <c r="B28" s="8">
-        <f>ROW(B28)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>26</v>
       </c>
       <c r="C28" s="12" t="s">
@@ -3170,7 +2577,7 @@
     <row r="29" spans="1:12">
       <c r="A29" s="3"/>
       <c r="B29" s="8">
-        <f>ROW(B29)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>27</v>
       </c>
       <c r="C29" s="9" t="s">
@@ -3200,10 +2607,10 @@
       <c r="K29" s="10"/>
       <c r="L29" s="10"/>
     </row>
-    <row r="30" ht="24.75" spans="1:12">
+    <row r="30" spans="1:12" ht="24">
       <c r="A30" s="3"/>
       <c r="B30" s="8">
-        <f>ROW(B30)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>28</v>
       </c>
       <c r="C30" s="12" t="s">
@@ -3233,10 +2640,10 @@
       <c r="K30" s="13"/>
       <c r="L30" s="13"/>
     </row>
-    <row r="31" spans="1:12">
+    <row r="31" spans="1:12" ht="24">
       <c r="A31" s="3"/>
       <c r="B31" s="8">
-        <f>ROW(B31)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>29</v>
       </c>
       <c r="C31" s="9" t="s">
@@ -3266,10 +2673,10 @@
       <c r="K31" s="10"/>
       <c r="L31" s="10"/>
     </row>
-    <row r="32" ht="36.75" spans="1:12">
+    <row r="32" spans="1:12" ht="36">
       <c r="A32" s="3"/>
       <c r="B32" s="8">
-        <f>ROW(B32)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>30</v>
       </c>
       <c r="C32" s="12" t="s">
@@ -3299,10 +2706,10 @@
       <c r="K32" s="13"/>
       <c r="L32" s="13"/>
     </row>
-    <row r="33" ht="24.75" spans="1:12">
+    <row r="33" spans="1:12" ht="24">
       <c r="A33" s="3"/>
       <c r="B33" s="8">
-        <f>ROW(B33)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>31</v>
       </c>
       <c r="C33" s="12" t="s">
@@ -3330,10 +2737,10 @@
       <c r="K33" s="10"/>
       <c r="L33" s="10"/>
     </row>
-    <row r="34" ht="36.75" spans="1:12">
+    <row r="34" spans="1:12" ht="36">
       <c r="A34" s="3"/>
       <c r="B34" s="8">
-        <f>ROW(B34)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="C34" s="12" t="s">
@@ -3363,10 +2770,10 @@
       <c r="K34" s="13"/>
       <c r="L34" s="13"/>
     </row>
-    <row r="35" ht="36.75" spans="1:12">
+    <row r="35" spans="1:12" ht="36">
       <c r="A35" s="3"/>
       <c r="B35" s="8">
-        <f>ROW(B35)-ROW($B$2)</f>
+        <f t="shared" ref="B35:B67" si="1">ROW(B35)-ROW($B$2)</f>
         <v>33</v>
       </c>
       <c r="C35" s="9" t="s">
@@ -3396,10 +2803,10 @@
       <c r="K35" s="10"/>
       <c r="L35" s="10"/>
     </row>
-    <row r="36" ht="36.75" spans="1:12">
+    <row r="36" spans="1:12" ht="36">
       <c r="A36" s="3"/>
       <c r="B36" s="8">
-        <f>ROW(B36)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>34</v>
       </c>
       <c r="C36" s="12" t="s">
@@ -3432,7 +2839,7 @@
     <row r="37" spans="1:12">
       <c r="A37" s="3"/>
       <c r="B37" s="8">
-        <f>ROW(B37)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>35</v>
       </c>
       <c r="C37" s="9" t="s">
@@ -3465,7 +2872,7 @@
     <row r="38" spans="1:12">
       <c r="A38" s="3"/>
       <c r="B38" s="8">
-        <f>ROW(B38)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>36</v>
       </c>
       <c r="C38" s="12" t="s">
@@ -3498,7 +2905,7 @@
     <row r="39" spans="1:12">
       <c r="A39" s="3"/>
       <c r="B39" s="8">
-        <f>ROW(B39)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>37</v>
       </c>
       <c r="C39" s="9" t="s">
@@ -3531,7 +2938,7 @@
     <row r="40" spans="1:12">
       <c r="A40" s="3"/>
       <c r="B40" s="8">
-        <f>ROW(B40)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>38</v>
       </c>
       <c r="C40" s="12" t="s">
@@ -3561,10 +2968,10 @@
       <c r="K40" s="13"/>
       <c r="L40" s="13"/>
     </row>
-    <row r="41" ht="15.75" spans="1:12">
+    <row r="41" spans="1:12">
       <c r="A41" s="3"/>
       <c r="B41" s="8">
-        <f>ROW(B41)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>39</v>
       </c>
       <c r="C41" s="9" t="s">
@@ -3594,10 +3001,10 @@
       <c r="K41" s="10"/>
       <c r="L41" s="10"/>
     </row>
-    <row r="42" ht="15.75" spans="1:12">
+    <row r="42" spans="1:12">
       <c r="A42" s="3"/>
       <c r="B42" s="8">
-        <f>ROW(B42)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>40</v>
       </c>
       <c r="C42" s="12" t="s">
@@ -3627,10 +3034,10 @@
       <c r="K42" s="13"/>
       <c r="L42" s="13"/>
     </row>
-    <row r="43" ht="36.75" spans="1:12">
+    <row r="43" spans="1:12" ht="36">
       <c r="A43" s="3"/>
       <c r="B43" s="8">
-        <f>ROW(B43)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>41</v>
       </c>
       <c r="C43" s="9" t="s">
@@ -3660,10 +3067,10 @@
       <c r="K43" s="10"/>
       <c r="L43" s="10"/>
     </row>
-    <row r="44" ht="36.75" spans="1:12">
+    <row r="44" spans="1:12" ht="36">
       <c r="A44" s="3"/>
       <c r="B44" s="8">
-        <f>ROW(B44)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>42</v>
       </c>
       <c r="C44" s="12" t="s">
@@ -3693,10 +3100,10 @@
       <c r="K44" s="13"/>
       <c r="L44" s="13"/>
     </row>
-    <row r="45" ht="36.75" spans="1:12">
+    <row r="45" spans="1:12" ht="36">
       <c r="A45" s="3"/>
       <c r="B45" s="8">
-        <f>ROW(B45)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>43</v>
       </c>
       <c r="C45" s="9" t="s">
@@ -3726,10 +3133,10 @@
       <c r="K45" s="10"/>
       <c r="L45" s="10"/>
     </row>
-    <row r="46" ht="24.75" spans="1:12">
+    <row r="46" spans="1:12" ht="24">
       <c r="A46" s="3"/>
       <c r="B46" s="8">
-        <f>ROW(B46)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>44</v>
       </c>
       <c r="C46" s="12" t="s">
@@ -3759,10 +3166,10 @@
       <c r="K46" s="13"/>
       <c r="L46" s="13"/>
     </row>
-    <row r="47" ht="24.75" spans="1:12">
+    <row r="47" spans="1:12" ht="24">
       <c r="A47" s="3"/>
       <c r="B47" s="8">
-        <f>ROW(B47)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>45</v>
       </c>
       <c r="C47" s="9" t="s">
@@ -3795,7 +3202,7 @@
     <row r="48" spans="1:12">
       <c r="A48" s="3"/>
       <c r="B48" s="8">
-        <f>ROW(B48)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>46</v>
       </c>
       <c r="C48" s="12" t="s">
@@ -3825,10 +3232,10 @@
       <c r="K48" s="13"/>
       <c r="L48" s="13"/>
     </row>
-    <row r="49" ht="36.75" spans="1:12">
+    <row r="49" spans="1:12" ht="36">
       <c r="A49" s="3"/>
       <c r="B49" s="8">
-        <f>ROW(B49)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>47</v>
       </c>
       <c r="C49" s="9" t="s">
@@ -3861,7 +3268,7 @@
     <row r="50" spans="1:12">
       <c r="A50" s="3"/>
       <c r="B50" s="8">
-        <f>ROW(B50)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>48</v>
       </c>
       <c r="C50" s="12" t="s">
@@ -3891,10 +3298,10 @@
       <c r="K50" s="13"/>
       <c r="L50" s="13"/>
     </row>
-    <row r="51" ht="24.75" spans="1:12">
+    <row r="51" spans="1:12" ht="24">
       <c r="A51" s="3"/>
       <c r="B51" s="8">
-        <f>ROW(B51)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>49</v>
       </c>
       <c r="C51" s="9" t="s">
@@ -3927,7 +3334,7 @@
     <row r="52" spans="1:12">
       <c r="A52" s="3"/>
       <c r="B52" s="8">
-        <f>ROW(B52)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>50</v>
       </c>
       <c r="C52" s="12" t="s">
@@ -3960,7 +3367,7 @@
     <row r="53" spans="1:12">
       <c r="A53" s="3"/>
       <c r="B53" s="8">
-        <f>ROW(B53)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>51</v>
       </c>
       <c r="C53" s="9" t="s">
@@ -3990,10 +3397,10 @@
       <c r="K53" s="10"/>
       <c r="L53" s="10"/>
     </row>
-    <row r="54" ht="36.75" spans="1:12">
+    <row r="54" spans="1:12" ht="36">
       <c r="A54" s="3"/>
       <c r="B54" s="8">
-        <f>ROW(B54)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>52</v>
       </c>
       <c r="C54" s="12" t="s">
@@ -4026,7 +3433,7 @@
     <row r="55" spans="1:12">
       <c r="A55" s="3"/>
       <c r="B55" s="8">
-        <f>ROW(B55)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>53</v>
       </c>
       <c r="C55" s="9" t="s">
@@ -4056,10 +3463,10 @@
       <c r="K55" s="10"/>
       <c r="L55" s="10"/>
     </row>
-    <row r="56" ht="24.75" spans="1:12">
+    <row r="56" spans="1:12" ht="24">
       <c r="A56" s="3"/>
       <c r="B56" s="8">
-        <f>ROW(B56)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>54</v>
       </c>
       <c r="C56" s="12" t="s">
@@ -4089,10 +3496,10 @@
       <c r="K56" s="13"/>
       <c r="L56" s="13"/>
     </row>
-    <row r="57" ht="24.75" spans="1:12">
+    <row r="57" spans="1:12" ht="24">
       <c r="A57" s="3"/>
       <c r="B57" s="8">
-        <f>ROW(B57)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>55</v>
       </c>
       <c r="C57" s="9" t="s">
@@ -4122,10 +3529,10 @@
       <c r="K57" s="10"/>
       <c r="L57" s="10"/>
     </row>
-    <row r="58" ht="24.75" spans="1:12">
+    <row r="58" spans="1:12" ht="24">
       <c r="A58" s="3"/>
       <c r="B58" s="8">
-        <f>ROW(B58)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>56</v>
       </c>
       <c r="C58" s="12" t="s">
@@ -4155,10 +3562,10 @@
       <c r="K58" s="13"/>
       <c r="L58" s="13"/>
     </row>
-    <row r="59" ht="24.75" spans="1:12">
+    <row r="59" spans="1:12" ht="24">
       <c r="A59" s="3"/>
       <c r="B59" s="8">
-        <f>ROW(B59)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>57</v>
       </c>
       <c r="C59" s="9" t="s">
@@ -4188,10 +3595,10 @@
       <c r="K59" s="10"/>
       <c r="L59" s="10"/>
     </row>
-    <row r="60" ht="24.75" spans="1:12">
+    <row r="60" spans="1:12" ht="36">
       <c r="A60" s="3"/>
       <c r="B60" s="8">
-        <f>ROW(B60)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>58</v>
       </c>
       <c r="C60" s="12" t="s">
@@ -4221,10 +3628,10 @@
       <c r="K60" s="13"/>
       <c r="L60" s="13"/>
     </row>
-    <row r="61" ht="36.75" spans="1:12">
+    <row r="61" spans="1:12" ht="36">
       <c r="A61" s="3"/>
       <c r="B61" s="8">
-        <f>ROW(B61)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>59</v>
       </c>
       <c r="C61" s="9" t="s">
@@ -4254,10 +3661,10 @@
       <c r="K61" s="10"/>
       <c r="L61" s="10"/>
     </row>
-    <row r="62" ht="24.75" spans="1:12">
+    <row r="62" spans="1:12" ht="24">
       <c r="A62" s="3"/>
       <c r="B62" s="8">
-        <f>ROW(B62)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>60</v>
       </c>
       <c r="C62" s="12" t="s">
@@ -4287,10 +3694,10 @@
       <c r="K62" s="13"/>
       <c r="L62" s="13"/>
     </row>
-    <row r="63" s="1" customFormat="1" ht="15.75" spans="1:12">
+    <row r="63" spans="1:12" s="1" customFormat="1">
       <c r="A63" s="17"/>
       <c r="B63" s="8">
-        <f>ROW(B63)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>61</v>
       </c>
       <c r="C63" s="12" t="s">
@@ -4315,13 +3722,13 @@
       <c r="J63" s="13">
         <v>1</v>
       </c>
-      <c r="K63" s="21"/>
-      <c r="L63" s="21"/>
-    </row>
-    <row r="64" s="1" customFormat="1" ht="15.75" spans="1:12">
+      <c r="K63" s="20"/>
+      <c r="L63" s="20"/>
+    </row>
+    <row r="64" spans="1:12" s="1" customFormat="1">
       <c r="A64" s="17"/>
       <c r="B64" s="8">
-        <f>ROW(B64)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>62</v>
       </c>
       <c r="C64" s="12" t="s">
@@ -4340,13 +3747,13 @@
       <c r="J64" s="13">
         <v>1</v>
       </c>
-      <c r="K64" s="22"/>
-      <c r="L64" s="22"/>
-    </row>
-    <row r="65" s="1" customFormat="1" ht="15.75" spans="1:12">
+      <c r="K64" s="21"/>
+      <c r="L64" s="21"/>
+    </row>
+    <row r="65" spans="1:13" s="1" customFormat="1">
       <c r="A65" s="17"/>
       <c r="B65" s="8">
-        <f>ROW(B65)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>63</v>
       </c>
       <c r="C65" s="12" t="s">
@@ -4365,13 +3772,13 @@
       <c r="J65" s="13">
         <v>1</v>
       </c>
-      <c r="K65" s="21"/>
-      <c r="L65" s="21"/>
-    </row>
-    <row r="66" s="1" customFormat="1" ht="15.75" spans="1:12">
+      <c r="K65" s="20"/>
+      <c r="L65" s="20"/>
+    </row>
+    <row r="66" spans="1:13" s="1" customFormat="1">
       <c r="A66" s="17"/>
       <c r="B66" s="8">
-        <f>ROW(B66)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>64</v>
       </c>
       <c r="C66" s="12" t="s">
@@ -4390,13 +3797,13 @@
       <c r="J66" s="13">
         <v>1</v>
       </c>
-      <c r="K66" s="21"/>
-      <c r="L66" s="21"/>
-    </row>
-    <row r="67" s="1" customFormat="1" ht="15.75" spans="1:12">
+      <c r="K66" s="20"/>
+      <c r="L66" s="20"/>
+    </row>
+    <row r="67" spans="1:13" s="1" customFormat="1" ht="30">
       <c r="A67" s="17"/>
       <c r="B67" s="8">
-        <f>ROW(B67)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>65</v>
       </c>
       <c r="C67" s="12" t="s">
@@ -4415,45 +3822,46 @@
       <c r="J67" s="13">
         <v>1</v>
       </c>
-      <c r="K67" s="21"/>
-      <c r="L67" s="21"/>
-    </row>
-    <row r="68" s="1" customFormat="1" spans="1:13">
+      <c r="K67" s="20"/>
+      <c r="L67" s="35" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="68" spans="1:13" s="1" customFormat="1">
       <c r="A68" s="17"/>
-      <c r="B68" s="23"/>
-      <c r="C68" s="24"/>
-      <c r="D68" s="25"/>
-      <c r="E68" s="26"/>
-      <c r="F68" s="27"/>
-      <c r="G68" s="28"/>
-      <c r="H68" s="27"/>
-      <c r="I68" s="28"/>
-      <c r="J68" s="28"/>
-      <c r="K68" s="28"/>
-      <c r="L68" s="28"/>
-      <c r="M68" s="33"/>
-    </row>
-    <row r="69" s="1" customFormat="1" ht="15.75" spans="1:13">
+      <c r="B68" s="22"/>
+      <c r="C68" s="23"/>
+      <c r="D68" s="24"/>
+      <c r="E68" s="25"/>
+      <c r="F68" s="26"/>
+      <c r="G68" s="27"/>
+      <c r="H68" s="26"/>
+      <c r="I68" s="27"/>
+      <c r="J68" s="27"/>
+      <c r="K68" s="27"/>
+      <c r="L68" s="27"/>
+      <c r="M68" s="32"/>
+    </row>
+    <row r="69" spans="1:13" s="1" customFormat="1">
       <c r="A69" s="17"/>
-      <c r="B69" s="29"/>
-      <c r="C69" s="30"/>
-      <c r="D69" s="31"/>
-      <c r="E69" s="32"/>
-      <c r="F69" s="32"/>
-      <c r="G69" s="32"/>
-      <c r="H69" s="32"/>
-      <c r="I69" s="32"/>
-      <c r="J69" s="32"/>
-      <c r="K69" s="32"/>
-      <c r="L69" s="32"/>
-      <c r="M69" s="34"/>
+      <c r="B69" s="28"/>
+      <c r="C69" s="29"/>
+      <c r="D69" s="30"/>
+      <c r="E69" s="31"/>
+      <c r="F69" s="31"/>
+      <c r="G69" s="31"/>
+      <c r="H69" s="31"/>
+      <c r="I69" s="31"/>
+      <c r="J69" s="31"/>
+      <c r="K69" s="31"/>
+      <c r="L69" s="31"/>
+      <c r="M69" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="I1:L1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>